<commit_message>
done with win 10 module vulnID updates
</commit_message>
<xml_diff>
--- a/vuln id update.xlsx
+++ b/vuln id update.xlsx
@@ -21,12 +21,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">map!$A$1:$F$286</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'vuln id update'!$A$1:$AN$286</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7716" uniqueCount="3042">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7695" uniqueCount="3021">
   <si>
     <t>TechnologyArea</t>
   </si>
@@ -12374,73 +12374,10 @@
     <t>220700</t>
   </si>
   <si>
-    <t>220879</t>
-  </si>
-  <si>
-    <t>220880</t>
-  </si>
-  <si>
-    <t>220881</t>
-  </si>
-  <si>
-    <t>220882</t>
-  </si>
-  <si>
-    <t>220883</t>
-  </si>
-  <si>
-    <t>220884</t>
-  </si>
-  <si>
-    <t>220885</t>
-  </si>
-  <si>
-    <t>220886</t>
-  </si>
-  <si>
-    <t>220887</t>
-  </si>
-  <si>
-    <t>220888</t>
-  </si>
-  <si>
-    <t>220889</t>
-  </si>
-  <si>
     <t>220890</t>
   </si>
   <si>
-    <t>220891</t>
-  </si>
-  <si>
-    <t>220893</t>
-  </si>
-  <si>
-    <t>220894</t>
-  </si>
-  <si>
     <t>220895</t>
-  </si>
-  <si>
-    <t>220896</t>
-  </si>
-  <si>
-    <t>220897</t>
-  </si>
-  <si>
-    <t>220898</t>
-  </si>
-  <si>
-    <t>220899</t>
-  </si>
-  <si>
-    <t>220900</t>
-  </si>
-  <si>
-    <t>220901</t>
-  </si>
-  <si>
-    <t>220704</t>
   </si>
   <si>
     <t>220872</t>
@@ -13272,7 +13209,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE286"/>
+  <dimension ref="A1:F286"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9" style="1" bestFit="1" customWidth="1"/>
@@ -19568,12 +19505,12 @@
         <v>2626</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>2627</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>3018</v>
+      <c r="B31" s="5">
+        <v>220879</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>1598</v>
@@ -19615,12 +19552,12 @@
         <v>2627</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="375" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" ht="375" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>2628</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>3019</v>
+      <c r="B32" s="5">
+        <v>220880</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>1605</v>
@@ -19662,12 +19599,12 @@
         <v>2628</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>2629</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>3020</v>
+      <c r="B33" s="5">
+        <v>220881</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>1612</v>
@@ -19709,12 +19646,12 @@
         <v>2629</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="405" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" ht="405" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>2630</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>3021</v>
+      <c r="B34" s="5">
+        <v>220882</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>1619</v>
@@ -19756,12 +19693,12 @@
         <v>2630</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>2631</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>3022</v>
+      <c r="B35" s="5">
+        <v>220883</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>1626</v>
@@ -19803,12 +19740,12 @@
         <v>2631</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>2632</v>
       </c>
-      <c r="B36" s="5" t="s">
-        <v>3023</v>
+      <c r="B36" s="5">
+        <v>220884</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>1633</v>
@@ -19850,12 +19787,12 @@
         <v>2632</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>2633</v>
       </c>
-      <c r="B37" s="5" t="s">
-        <v>3024</v>
+      <c r="B37" s="5">
+        <v>220885</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>1640</v>
@@ -19897,12 +19834,12 @@
         <v>2633</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>2634</v>
       </c>
-      <c r="B38" s="5" t="s">
-        <v>3025</v>
+      <c r="B38" s="5">
+        <v>220886</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>1647</v>
@@ -19944,12 +19881,12 @@
         <v>2634</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>2635</v>
       </c>
-      <c r="B39" s="5" t="s">
-        <v>3026</v>
+      <c r="B39" s="5">
+        <v>220887</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>1654</v>
@@ -19991,12 +19928,12 @@
         <v>2635</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>2636</v>
       </c>
-      <c r="B40" s="5" t="s">
-        <v>3027</v>
+      <c r="B40" s="5">
+        <v>220888</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>1661</v>
@@ -20038,12 +19975,12 @@
         <v>2636</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>2637</v>
       </c>
-      <c r="B41" s="5" t="s">
-        <v>3028</v>
+      <c r="B41" s="5">
+        <v>220889</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>1668</v>
@@ -20085,12 +20022,12 @@
         <v>2637</v>
       </c>
     </row>
-    <row r="42" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>2638</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>3029</v>
+        <v>3018</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>1675</v>
@@ -20132,12 +20069,12 @@
         <v>2638</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>2639</v>
       </c>
-      <c r="B43" s="5" t="s">
-        <v>3030</v>
+      <c r="B43" s="5">
+        <v>220891</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>1682</v>
@@ -20179,12 +20116,12 @@
         <v>2639</v>
       </c>
     </row>
-    <row r="44" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>2640</v>
       </c>
-      <c r="B44" s="5" t="s">
-        <v>3031</v>
+      <c r="B44" s="5">
+        <v>220893</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>1689</v>
@@ -20226,12 +20163,12 @@
         <v>2640</v>
       </c>
     </row>
-    <row r="45" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>2641</v>
       </c>
-      <c r="B45" s="5" t="s">
-        <v>3032</v>
+      <c r="B45" s="5">
+        <v>220894</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>1696</v>
@@ -20273,12 +20210,12 @@
         <v>2641</v>
       </c>
     </row>
-    <row r="46" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>2642</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>3033</v>
+        <v>3019</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>1703</v>
@@ -20320,12 +20257,12 @@
         <v>2642</v>
       </c>
     </row>
-    <row r="47" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>2643</v>
       </c>
-      <c r="B47" s="5" t="s">
-        <v>3034</v>
+      <c r="B47" s="5">
+        <v>220896</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>1710</v>
@@ -20367,12 +20304,12 @@
         <v>2643</v>
       </c>
     </row>
-    <row r="48" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>2644</v>
       </c>
-      <c r="B48" s="5" t="s">
-        <v>3035</v>
+      <c r="B48" s="5">
+        <v>220897</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>1717</v>
@@ -20414,12 +20351,12 @@
         <v>2644</v>
       </c>
     </row>
-    <row r="49" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>2645</v>
       </c>
-      <c r="B49" s="5" t="s">
-        <v>3036</v>
+      <c r="B49" s="5">
+        <v>220898</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>1724</v>
@@ -20461,12 +20398,12 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="50" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>2646</v>
       </c>
-      <c r="B50" s="5" t="s">
-        <v>3037</v>
+      <c r="B50" s="5">
+        <v>220899</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>1731</v>
@@ -20508,12 +20445,12 @@
         <v>2646</v>
       </c>
     </row>
-    <row r="51" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>2647</v>
       </c>
-      <c r="B51" s="5" t="s">
-        <v>3038</v>
+      <c r="B51" s="5">
+        <v>220900</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>1738</v>
@@ -20555,12 +20492,12 @@
         <v>2647</v>
       </c>
     </row>
-    <row r="52" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>2648</v>
       </c>
-      <c r="B52" s="5" t="s">
-        <v>3039</v>
+      <c r="B52" s="5">
+        <v>220901</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>1745</v>
@@ -20602,12 +20539,12 @@
         <v>2648</v>
       </c>
     </row>
-    <row r="53" spans="1:16" ht="240" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" ht="240" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>2453</v>
       </c>
-      <c r="B53" s="5" t="s">
-        <v>3040</v>
+      <c r="B53" s="5">
+        <v>220704</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>107</v>
@@ -20654,7 +20591,7 @@
         <v>2620</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>3041</v>
+        <v>3020</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>1542</v>
@@ -20704,43 +20641,40 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AN286"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="6.28515625" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" style="1" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="6.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" style="1" customWidth="1"/>
     <col min="7" max="7" width="11.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.42578125" style="1" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="26.140625" style="1" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="26.140625" style="1" customWidth="1"/>
     <col min="10" max="10" width="25.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.42578125" style="1" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="16.42578125" style="1" customWidth="1"/>
     <col min="12" max="12" width="153.42578125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="28" style="1" customWidth="1"/>
-    <col min="14" max="14" width="28" style="1" hidden="1" customWidth="1"/>
-    <col min="15" max="16" width="28" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.140625" style="1" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="15" style="1" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="14.140625" style="1" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="11" style="1" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="15.7109375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="15.85546875" style="1" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="17.42578125" style="1" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="13.7109375" style="1" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="25.85546875" style="1" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="23.85546875" style="1" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="12.7109375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="16" width="28" style="1" customWidth="1"/>
+    <col min="17" max="17" width="14.140625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="15" style="1" customWidth="1"/>
+    <col min="19" max="19" width="14.140625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11" style="1" customWidth="1"/>
+    <col min="21" max="21" width="15.7109375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="15.85546875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="17.42578125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="13.7109375" style="1" customWidth="1"/>
+    <col min="25" max="25" width="25.85546875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="23.85546875" style="1" customWidth="1"/>
+    <col min="27" max="27" width="12.7109375" style="1" customWidth="1"/>
     <col min="28" max="28" width="98.28515625" style="1" customWidth="1"/>
     <col min="29" max="29" width="13.7109375" style="1" customWidth="1"/>
-    <col min="30" max="30" width="10.5703125" style="1" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="14.28515625" style="1" hidden="1" customWidth="1"/>
-    <col min="32" max="32" width="16.7109375" style="1" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="28.28515625" style="1" hidden="1" customWidth="1"/>
-    <col min="34" max="34" width="99.42578125" style="1" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="10.5703125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="14.28515625" style="1" customWidth="1"/>
+    <col min="32" max="32" width="16.7109375" style="1" customWidth="1"/>
+    <col min="33" max="33" width="28.28515625" style="1" customWidth="1"/>
+    <col min="34" max="34" width="99.42578125" style="1" customWidth="1"/>
     <col min="35" max="35" width="27.5703125" style="1" customWidth="1"/>
     <col min="36" max="36" width="36" style="1" customWidth="1"/>
     <col min="37" max="38" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -20869,7 +20803,7 @@
         <v>3016</v>
       </c>
     </row>
-    <row r="2" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2446</v>
       </c>
@@ -21005,7 +20939,7 @@
         <v>V-100093</v>
       </c>
     </row>
-    <row r="4" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2448</v>
       </c>
@@ -21141,7 +21075,7 @@
         <v>V-63323</v>
       </c>
     </row>
-    <row r="6" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>2450</v>
       </c>
@@ -21207,7 +21141,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>2451</v>
       </c>
@@ -21273,7 +21207,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="8" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2452</v>
       </c>
@@ -21479,7 +21413,7 @@
         <v>V-63351</v>
       </c>
     </row>
-    <row r="11" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>2455</v>
       </c>
@@ -21615,7 +21549,7 @@
         <v>V-63355</v>
       </c>
     </row>
-    <row r="13" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2457</v>
       </c>
@@ -22031,7 +21965,7 @@
         <v>V-63367</v>
       </c>
     </row>
-    <row r="19" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>2463</v>
       </c>
@@ -22237,7 +22171,7 @@
         <v>V-63393</v>
       </c>
     </row>
-    <row r="22" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>2466</v>
       </c>
@@ -22303,7 +22237,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="23" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>2467</v>
       </c>
@@ -22369,7 +22303,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="24" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>2468</v>
       </c>
@@ -22435,7 +22369,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="25" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>2469</v>
       </c>
@@ -22501,7 +22435,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="26" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>2470</v>
       </c>
@@ -22567,7 +22501,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="27" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>2471</v>
       </c>
@@ -22773,7 +22707,7 @@
         <v>V-63545</v>
       </c>
     </row>
-    <row r="30" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>2474</v>
       </c>
@@ -22909,7 +22843,7 @@
         <v>V-63587</v>
       </c>
     </row>
-    <row r="32" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>2476</v>
       </c>
@@ -22975,7 +22909,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="33" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>2477</v>
       </c>
@@ -23041,7 +22975,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="34" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>2478</v>
       </c>
@@ -23107,7 +23041,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="35" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>2479</v>
       </c>
@@ -23173,7 +23107,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="36" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>2480</v>
       </c>
@@ -23239,7 +23173,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="37" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>2481</v>
       </c>
@@ -23375,7 +23309,7 @@
         <v>V-63595</v>
       </c>
     </row>
-    <row r="39" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>2483</v>
       </c>
@@ -23441,7 +23375,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="40" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>2484</v>
       </c>
@@ -23507,7 +23441,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="41" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>2485</v>
       </c>
@@ -23573,7 +23507,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="42" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>2486</v>
       </c>
@@ -23639,7 +23573,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="43" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>2487</v>
       </c>
@@ -23705,7 +23639,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="44" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>2488</v>
       </c>
@@ -23771,7 +23705,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="45" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>2489</v>
       </c>
@@ -23837,7 +23771,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="46" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>2490</v>
       </c>
@@ -23903,7 +23837,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="47" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>2491</v>
       </c>
@@ -23969,7 +23903,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="48" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>2492</v>
       </c>
@@ -24035,7 +23969,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="49" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>2493</v>
       </c>
@@ -24101,7 +24035,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="50" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>2494</v>
       </c>
@@ -24167,7 +24101,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="51" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>2495</v>
       </c>
@@ -24233,7 +24167,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="52" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>2496</v>
       </c>
@@ -24299,7 +24233,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="53" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>2497</v>
       </c>
@@ -24365,7 +24299,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="54" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>2498</v>
       </c>
@@ -24431,7 +24365,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="55" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>2499</v>
       </c>
@@ -24497,7 +24431,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="56" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>2500</v>
       </c>
@@ -24563,7 +24497,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="57" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>2501</v>
       </c>
@@ -24629,7 +24563,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="58" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>2502</v>
       </c>
@@ -24695,7 +24629,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="59" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>2503</v>
       </c>
@@ -24761,7 +24695,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="60" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>2504</v>
       </c>
@@ -24827,7 +24761,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="61" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>2505</v>
       </c>
@@ -24893,7 +24827,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="62" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>2506</v>
       </c>
@@ -24959,7 +24893,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="63" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>2507</v>
       </c>
@@ -25025,7 +24959,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="64" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>2508</v>
       </c>
@@ -25091,7 +25025,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="65" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>2509</v>
       </c>
@@ -25157,7 +25091,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="66" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>2510</v>
       </c>
@@ -25223,7 +25157,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="67" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>2511</v>
       </c>
@@ -25289,7 +25223,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="68" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>2512</v>
       </c>
@@ -25355,7 +25289,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="69" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>2513</v>
       </c>
@@ -25421,7 +25355,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="70" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>2514</v>
       </c>
@@ -25487,7 +25421,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="71" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>2515</v>
       </c>
@@ -25553,7 +25487,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="72" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>2516</v>
       </c>
@@ -25619,7 +25553,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="73" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>2517</v>
       </c>
@@ -25685,7 +25619,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="74" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>2518</v>
       </c>
@@ -25751,7 +25685,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="75" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>2519</v>
       </c>
@@ -25817,7 +25751,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="76" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>2520</v>
       </c>
@@ -25883,7 +25817,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="77" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>2521</v>
       </c>
@@ -25949,7 +25883,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="78" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>2522</v>
       </c>
@@ -26015,7 +25949,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="79" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>2523</v>
       </c>
@@ -26081,7 +26015,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="80" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>2524</v>
       </c>
@@ -26147,7 +26081,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="81" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>2525</v>
       </c>
@@ -26213,7 +26147,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="82" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>2526</v>
       </c>
@@ -26279,7 +26213,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="83" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>2527</v>
       </c>
@@ -26345,7 +26279,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="84" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>2528</v>
       </c>
@@ -26411,7 +26345,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="85" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>2529</v>
       </c>
@@ -26477,7 +26411,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="86" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>2530</v>
       </c>
@@ -26543,7 +26477,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="87" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>2531</v>
       </c>
@@ -26609,7 +26543,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="88" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>2532</v>
       </c>
@@ -26675,7 +26609,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="89" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>2533</v>
       </c>
@@ -26741,7 +26675,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="90" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>2534</v>
       </c>
@@ -26807,7 +26741,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="91" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>2535</v>
       </c>
@@ -26873,7 +26807,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="92" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>2536</v>
       </c>
@@ -26939,7 +26873,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="93" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>2537</v>
       </c>
@@ -27005,7 +26939,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="94" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>2538</v>
       </c>
@@ -27071,7 +27005,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="95" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>2539</v>
       </c>
@@ -27137,7 +27071,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="96" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>2540</v>
       </c>
@@ -27343,7 +27277,7 @@
         <v>V-63685</v>
       </c>
     </row>
-    <row r="99" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>2543</v>
       </c>
@@ -27409,7 +27343,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="100" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>2544</v>
       </c>
@@ -27475,7 +27409,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="101" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>2545</v>
       </c>
@@ -27541,7 +27475,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="102" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>2546</v>
       </c>
@@ -27607,7 +27541,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="103" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>2547</v>
       </c>
@@ -27673,7 +27607,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="104" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>2548</v>
       </c>
@@ -27739,7 +27673,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="105" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>2549</v>
       </c>
@@ -27805,7 +27739,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="106" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>2550</v>
       </c>
@@ -27871,7 +27805,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="107" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>2551</v>
       </c>
@@ -27937,7 +27871,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="108" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>2552</v>
       </c>
@@ -28003,7 +27937,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="109" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>2553</v>
       </c>
@@ -28139,7 +28073,7 @@
         <v>V-63739</v>
       </c>
     </row>
-    <row r="111" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>2555</v>
       </c>
@@ -28205,7 +28139,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="112" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>2556</v>
       </c>
@@ -28271,7 +28205,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="113" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>2557</v>
       </c>
@@ -28337,7 +28271,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="114" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>2558</v>
       </c>
@@ -28403,7 +28337,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="115" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>2559</v>
       </c>
@@ -28609,7 +28543,7 @@
         <v>V-74413</v>
       </c>
     </row>
-    <row r="118" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>2562</v>
       </c>
@@ -28675,7 +28609,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="119" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>2563</v>
       </c>
@@ -28741,7 +28675,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="120" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>2564</v>
       </c>
@@ -28807,7 +28741,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="121" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>2565</v>
       </c>
@@ -28873,7 +28807,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="122" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>2566</v>
       </c>
@@ -28939,7 +28873,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="123" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>2567</v>
       </c>
@@ -29005,7 +28939,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="124" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>2568</v>
       </c>
@@ -29071,7 +29005,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="125" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>2569</v>
       </c>
@@ -29137,7 +29071,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="126" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>2570</v>
       </c>
@@ -29203,7 +29137,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="127" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>2571</v>
       </c>
@@ -29269,7 +29203,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="128" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>2572</v>
       </c>
@@ -29335,7 +29269,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="129" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>2573</v>
       </c>
@@ -29401,7 +29335,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="130" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>2574</v>
       </c>
@@ -29467,7 +29401,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="131" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>2575</v>
       </c>
@@ -29533,7 +29467,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="132" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>2576</v>
       </c>
@@ -29599,7 +29533,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="133" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>2577</v>
       </c>
@@ -29665,7 +29599,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="134" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>2578</v>
       </c>
@@ -29731,7 +29665,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="135" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>2579</v>
       </c>
@@ -29797,7 +29731,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="136" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>2580</v>
       </c>
@@ -29863,7 +29797,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="137" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>2581</v>
       </c>
@@ -29929,7 +29863,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="138" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>2582</v>
       </c>
@@ -29995,7 +29929,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="139" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>2583</v>
       </c>
@@ -30061,7 +29995,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="140" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>2584</v>
       </c>
@@ -30197,7 +30131,7 @@
         <v>V-76505</v>
       </c>
     </row>
-    <row r="142" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>2586</v>
       </c>
@@ -30263,7 +30197,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="143" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>2587</v>
       </c>
@@ -30329,7 +30263,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="144" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>2588</v>
       </c>
@@ -30395,7 +30329,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="145" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>2589</v>
       </c>
@@ -30461,7 +30395,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="146" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>2590</v>
       </c>
@@ -30527,7 +30461,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="147" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>2591</v>
       </c>
@@ -30593,7 +30527,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="148" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>2592</v>
       </c>
@@ -30659,7 +30593,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="149" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>2593</v>
       </c>
@@ -30725,7 +30659,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="150" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>2594</v>
       </c>
@@ -30791,7 +30725,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="151" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>2595</v>
       </c>
@@ -30857,7 +30791,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="152" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>2596</v>
       </c>
@@ -30923,7 +30857,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="153" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>2597</v>
       </c>
@@ -30989,7 +30923,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="154" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>2598</v>
       </c>
@@ -31055,7 +30989,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="155" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>2599</v>
       </c>
@@ -31121,7 +31055,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="156" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>2600</v>
       </c>
@@ -31187,7 +31121,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="157" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>2601</v>
       </c>
@@ -31253,7 +31187,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="158" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>2602</v>
       </c>
@@ -31319,7 +31253,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="159" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>2603</v>
       </c>
@@ -31385,7 +31319,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="160" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>2604</v>
       </c>
@@ -31451,7 +31385,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="161" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>2605</v>
       </c>
@@ -31517,7 +31451,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="162" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>2606</v>
       </c>
@@ -31583,7 +31517,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="163" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>2607</v>
       </c>
@@ -31649,7 +31583,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="164" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>2608</v>
       </c>
@@ -31715,7 +31649,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="165" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>2609</v>
       </c>
@@ -31781,7 +31715,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="166" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>2610</v>
       </c>
@@ -31847,7 +31781,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="167" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>2611</v>
       </c>
@@ -31913,7 +31847,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="168" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>2612</v>
       </c>
@@ -31979,7 +31913,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="169" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>2613</v>
       </c>
@@ -32045,7 +31979,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="170" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>2614</v>
       </c>
@@ -32111,7 +32045,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="171" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>2615</v>
       </c>
@@ -32177,7 +32111,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="172" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>2616</v>
       </c>
@@ -32243,7 +32177,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="173" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>2617</v>
       </c>
@@ -32309,7 +32243,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="174" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>2618</v>
       </c>
@@ -32375,7 +32309,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="175" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>2619</v>
       </c>
@@ -34471,7 +34405,7 @@
         <v>V-77269</v>
       </c>
     </row>
-    <row r="205" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
         <v>2649</v>
       </c>
@@ -34537,7 +34471,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="206" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
         <v>2650</v>
       </c>
@@ -34603,7 +34537,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="207" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>2651</v>
       </c>
@@ -34739,7 +34673,7 @@
         <v>V-94861</v>
       </c>
     </row>
-    <row r="209" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
         <v>2653</v>
       </c>
@@ -34805,7 +34739,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="210" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>2654</v>
       </c>
@@ -34871,7 +34805,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="211" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
         <v>2655</v>
       </c>
@@ -34937,7 +34871,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="212" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
         <v>2656</v>
       </c>
@@ -35003,7 +34937,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="213" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
         <v>2657</v>
       </c>
@@ -35069,7 +35003,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="214" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
         <v>2658</v>
       </c>
@@ -35135,7 +35069,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="215" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>2659</v>
       </c>
@@ -35201,7 +35135,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="216" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>2660</v>
       </c>
@@ -35267,7 +35201,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="217" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
         <v>2661</v>
       </c>
@@ -35333,7 +35267,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="218" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>2662</v>
       </c>
@@ -35399,7 +35333,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="219" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
         <v>2663</v>
       </c>
@@ -35465,7 +35399,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="220" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>2664</v>
       </c>
@@ -35531,7 +35465,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="221" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
         <v>2665</v>
       </c>
@@ -35597,7 +35531,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="222" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
         <v>2666</v>
       </c>
@@ -35663,7 +35597,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="223" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
         <v>2667</v>
       </c>
@@ -35729,7 +35663,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="224" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
         <v>2668</v>
       </c>
@@ -35795,7 +35729,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="225" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
         <v>2669</v>
       </c>
@@ -35861,7 +35795,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="226" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
         <v>2670</v>
       </c>
@@ -35927,7 +35861,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="227" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
         <v>2671</v>
       </c>
@@ -35993,7 +35927,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="228" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
         <v>2672</v>
       </c>
@@ -36059,7 +35993,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="229" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
         <v>2673</v>
       </c>
@@ -36125,7 +36059,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="230" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
         <v>2674</v>
       </c>
@@ -36261,7 +36195,7 @@
         <v>V-99563</v>
       </c>
     </row>
-    <row r="232" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
         <v>2676</v>
       </c>
@@ -36327,7 +36261,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="233" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A233" s="1" t="s">
         <v>2677</v>
       </c>
@@ -36393,7 +36327,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="234" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
         <v>2678</v>
       </c>
@@ -36459,7 +36393,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="235" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A235" s="1" t="s">
         <v>2679</v>
       </c>
@@ -36525,7 +36459,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="236" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A236" s="1" t="s">
         <v>2680</v>
       </c>
@@ -36591,7 +36525,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="237" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A237" s="1" t="s">
         <v>2681</v>
       </c>
@@ -36657,7 +36591,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="238" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A238" s="1" t="s">
         <v>2682</v>
       </c>
@@ -36723,7 +36657,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="239" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A239" s="1" t="s">
         <v>2683</v>
       </c>
@@ -36789,7 +36723,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="240" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A240" s="1" t="s">
         <v>2684</v>
       </c>
@@ -36855,7 +36789,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="241" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
         <v>2685</v>
       </c>
@@ -36921,7 +36855,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="242" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A242" s="1" t="s">
         <v>2686</v>
       </c>
@@ -36987,7 +36921,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="243" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A243" s="1" t="s">
         <v>2687</v>
       </c>
@@ -37053,7 +36987,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="244" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A244" s="1" t="s">
         <v>2688</v>
       </c>
@@ -37119,7 +37053,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="245" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
         <v>2689</v>
       </c>
@@ -37185,7 +37119,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="246" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A246" s="1" t="s">
         <v>2690</v>
       </c>
@@ -37251,7 +37185,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="247" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A247" s="1" t="s">
         <v>2691</v>
       </c>
@@ -37317,7 +37251,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="248" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A248" s="1" t="s">
         <v>2692</v>
       </c>
@@ -37383,7 +37317,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="249" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A249" s="1" t="s">
         <v>2693</v>
       </c>
@@ -37449,7 +37383,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="250" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
         <v>2694</v>
       </c>
@@ -37515,7 +37449,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="251" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
         <v>2695</v>
       </c>
@@ -37581,7 +37515,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="252" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A252" s="1" t="s">
         <v>2696</v>
       </c>
@@ -37647,7 +37581,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="253" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A253" s="1" t="s">
         <v>2697</v>
       </c>
@@ -37713,7 +37647,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="254" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A254" s="1" t="s">
         <v>2698</v>
       </c>
@@ -37779,7 +37713,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="255" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A255" s="1" t="s">
         <v>2699</v>
       </c>
@@ -37845,7 +37779,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="256" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A256" s="1" t="s">
         <v>2700</v>
       </c>
@@ -37911,7 +37845,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="257" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A257" s="1" t="s">
         <v>2701</v>
       </c>
@@ -37977,7 +37911,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="258" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A258" s="1" t="s">
         <v>2702</v>
       </c>
@@ -38043,7 +37977,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="259" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A259" s="1" t="s">
         <v>2703</v>
       </c>
@@ -38109,7 +38043,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="260" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A260" s="1" t="s">
         <v>2704</v>
       </c>
@@ -38175,7 +38109,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="261" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A261" s="1" t="s">
         <v>2705</v>
       </c>
@@ -38241,7 +38175,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="262" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A262" s="1" t="s">
         <v>2706</v>
       </c>
@@ -38307,7 +38241,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="263" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
         <v>2707</v>
       </c>
@@ -38373,7 +38307,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="264" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A264" s="1" t="s">
         <v>2708</v>
       </c>
@@ -38439,7 +38373,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="265" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A265" s="1" t="s">
         <v>2709</v>
       </c>
@@ -38505,7 +38439,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="266" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
         <v>2710</v>
       </c>
@@ -38571,7 +38505,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="267" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
         <v>2711</v>
       </c>
@@ -38637,7 +38571,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="268" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
         <v>2712</v>
       </c>
@@ -38703,7 +38637,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="269" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
         <v>2713</v>
       </c>
@@ -38769,7 +38703,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="270" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A270" s="1" t="s">
         <v>2714</v>
       </c>
@@ -38835,7 +38769,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="271" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A271" s="1" t="s">
         <v>2715</v>
       </c>
@@ -38901,7 +38835,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="272" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
         <v>2716</v>
       </c>
@@ -38967,7 +38901,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="273" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A273" s="1" t="s">
         <v>2717</v>
       </c>
@@ -39033,7 +38967,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="274" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
         <v>2718</v>
       </c>
@@ -39099,7 +39033,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="275" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
         <v>2719</v>
       </c>
@@ -39165,7 +39099,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="276" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
         <v>2720</v>
       </c>
@@ -39231,7 +39165,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="277" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
         <v>2721</v>
       </c>
@@ -39297,7 +39231,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="278" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A278" s="1" t="s">
         <v>2722</v>
       </c>
@@ -39363,7 +39297,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="279" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
         <v>2723</v>
       </c>
@@ -39429,7 +39363,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="280" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
         <v>2724</v>
       </c>
@@ -39495,7 +39429,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="281" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
         <v>2725</v>
       </c>
@@ -39561,7 +39495,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="282" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
         <v>2726</v>
       </c>
@@ -39627,7 +39561,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="283" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
         <v>2727</v>
       </c>
@@ -39693,7 +39627,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="284" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
         <v>2728</v>
       </c>
@@ -39759,7 +39693,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="285" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
         <v>2729</v>
       </c>
@@ -39825,7 +39759,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="286" spans="1:40" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:40" x14ac:dyDescent="0.25">
       <c r="G286" s="1" t="s">
         <v>2437</v>
       </c>
@@ -39880,68 +39814,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN286">
-    <filterColumn colId="39">
-      <filters>
-        <filter val="V-100093"/>
-        <filter val="V-63323"/>
-        <filter val="V-63345"/>
-        <filter val="V-63351"/>
-        <filter val="V-63355"/>
-        <filter val="V-63357"/>
-        <filter val="V-63359"/>
-        <filter val="V-63361"/>
-        <filter val="V-63363"/>
-        <filter val="V-63367"/>
-        <filter val="V-63371"/>
-        <filter val="V-63393"/>
-        <filter val="V-63399"/>
-        <filter val="V-63545"/>
-        <filter val="V-63587"/>
-        <filter val="V-63595"/>
-        <filter val="V-63599"/>
-        <filter val="V-63685"/>
-        <filter val="V-63739"/>
-        <filter val="V-68845"/>
-        <filter val="V-74413"/>
-        <filter val="V-76505"/>
-        <filter val="V-77085"/>
-        <filter val="V-77091"/>
-        <filter val="V-77095"/>
-        <filter val="V-77097"/>
-        <filter val="V-77101"/>
-        <filter val="V-77103"/>
-        <filter val="V-77189"/>
-        <filter val="V-77191"/>
-        <filter val="V-77195"/>
-        <filter val="V-77201"/>
-        <filter val="V-77205"/>
-        <filter val="V-77209"/>
-        <filter val="V-77213"/>
-        <filter val="V-77217"/>
-        <filter val="V-77221"/>
-        <filter val="V-77223"/>
-        <filter val="V-77227"/>
-        <filter val="V-77231"/>
-        <filter val="V-77233"/>
-        <filter val="V-77239"/>
-        <filter val="V-77243"/>
-        <filter val="V-77245"/>
-        <filter val="V-77247"/>
-        <filter val="V-77249"/>
-        <filter val="V-77255"/>
-        <filter val="V-77259"/>
-        <filter val="V-77263"/>
-        <filter val="V-77267"/>
-        <filter val="V-77269"/>
-        <filter val="V-94861"/>
-        <filter val="V-99563"/>
-      </filters>
-    </filterColumn>
-    <sortState ref="A3:AM231">
-      <sortCondition ref="A1:A286"/>
-    </sortState>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>